<commit_message>
Rewrite additional steps following 書き方 format rules
分岐を「○○の場合→手順【N】へ」文章形式で記述、色なし白黒、
フォントHGP創英角ゴシックUB(本文24pt/補足16pt/急所14pt)に準拠。

https://claude.ai/code/session_014LN5dU5LtPSyG4iXygZNs3
</commit_message>
<xml_diff>
--- a/本文FMT_追加手順15-19.xlsx
+++ b/本文FMT_追加手順15-19.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="本文FMT (追加手順)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="本文FMT (例外処理手順)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,10 +26,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
+      <name val="HGP創英角ｺﾞｼｯｸUB"/>
       <color rgb="00C00000"/>
-      <sz val="10"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Arial Black"/>
@@ -37,7 +36,7 @@
     </font>
     <font>
       <name val="HGP創英角ｺﾞｼｯｸUB"/>
-      <sz val="20"/>
+      <sz val="24"/>
     </font>
     <font>
       <name val="HGP創英角ｺﾞｼｯｸUB"/>
@@ -48,36 +47,12 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-        <bgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E4DFEC"/>
-        <bgColor rgb="00E4DFEC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -89,44 +64,30 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
     <border>
-      <left style="hair">
-        <color rgb="00808080"/>
-      </left>
-      <right style="hair">
-        <color rgb="00808080"/>
-      </right>
-      <top style="hair">
-        <color rgb="00808080"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00808080"/>
-      </bottom>
+      <left style="hair"/>
+      <right style="hair"/>
+      <top style="hair"/>
+      <bottom style="hair"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,48 +98,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -255,36 +180,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>2</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3619500" cy="4324350"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -595,10 +490,16 @@
     <col width="9.33" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1" ht="130" customHeight="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>※元ファイル「本文FMT」シートの手順14の下(203行目以降)に、この行ごとコピー＆貼り付けしてください</t>
+          <t>【元ファイル 手順1 の「補足」欄(C14:H19)に追記する文章案】
+・LPN分割を実施した場合　　　　　→手順【15】へ
+・LPN分割を実施していない場合　　→手順【16】へ
+・LPN分割で数量を誤った場合　　　→手順【15】へ
+・LPN分割を過剰に行った場合　　　→手順【17】へ
+・複数部材のLPN分割を途中で中断した場合　→手順【18】へ
+・プリンタを設定しないままLPN分割した場合→手順【19】へ</t>
         </is>
       </c>
     </row>
@@ -610,8 +511,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>OLPN統合を実施する
-（①即出荷後にLPN分割した場合のYES分岐／②LPN分割で数量を誤った場合に対応）</t>
+          <t>OLPNを統合する</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr"/>
@@ -622,7 +522,7 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>統合対象のLPNを誤らないよう、現品票で再確認する</t>
+          <t>統合対象のLPNを現品票で再確認する</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr"/>
@@ -637,7 +537,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>統合先LPNの誤りによる出荷誤り防止</t>
+          <t>統合先LPN誤りによる出荷誤り防止</t>
         </is>
       </c>
     </row>
@@ -651,12 +551,9 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>【場合分け対応表】
-①即出荷後にLPN分割を忘れた → 手順15・16
-②LPN分割で数量を誤った　　　 → 手順15
-③LPN分割を過剰に行った　　　 → 手順17
-④複数部材のLPN分割を中断した → 手順18
-⑤プリンタ未設定のままLPN分割 → 手順19</t>
+          <t>対象：
+①即出荷後にLPN分割を実施した場合
+②LPN分割で数量を誤ってしまった場合</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -694,10 +591,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>対象がワンレックか確認し、梱包を実施する
-（①即出荷後にLPN分割していない場合のNO分岐）
-・ワンレック　→ 国内梱包（ワンレック）を実施する
-・複数レック　→ 国内梱包（複数レック）を実施し、イレギュラー置場へ移動する</t>
+          <t>対象がワンレックか確認し、梱包を実施する</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
@@ -708,7 +602,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>複数レックの場合、すべてのレックを移動したか確認する</t>
+          <t>複数レックの場合、全レック分を移動したか確認する</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr"/>
@@ -737,7 +631,12 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>複数レックの場合はイレギュラー置場への移動が必要。対応漏れがないよう関係者へ必ず周知すること。</t>
+          <t>対象：①即出荷後にLPN分割を実施しなかった場合
+・ワンレックの場合
+　→国内梱包（ワンレック）を実施する
+・複数レックの場合
+　→国内梱包（複数レック）を実施し、
+　　イレギュラー置場へ移動する</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -768,15 +667,14 @@
     <row r="25" ht="24" customHeight="1"/>
     <row r="26" ht="24" customHeight="1"/>
     <row r="27" ht="24" customHeight="1">
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>【③対応】分割ラベルを使用する
-LPN分割を過剰に行った場合、余分に発行されたラベルは「分割ラベル」として保管し、該当LPNに使用する。</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>分割ラベルを使用する</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr"/>
@@ -787,7 +685,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>誤って別LPNに分割ラベルを貼付しないよう、ラベルのLPN番号を必ず確認する</t>
+          <t>別LPNへの誤貼付防止のため、ラベルのLPN番号を必ず確認する</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr"/>
@@ -809,14 +707,17 @@
     <row r="31" ht="24" customHeight="1"/>
     <row r="32" ht="24" customHeight="1"/>
     <row r="33" ht="24" customHeight="1">
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>補足:</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>余分に発行したラベルは捨てずに保管箱へ入れること。</t>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>対象：③LPN分割を過剰に行った場合
+余分に発行されたラベルは「分割ラベル」として
+保管し、該当LPNに使用する。
+余分なラベルは捨てずに保管箱へ入れること。</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
@@ -839,15 +740,14 @@
     <row r="37" ht="24" customHeight="1"/>
     <row r="38" ht="24" customHeight="1"/>
     <row r="39" ht="24" customHeight="1">
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>【④対応】親部材集約を実施する
-複数部材のLPN分割作業を中断した場合、未処理の部材を親部材へ集約する。</t>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>親部材集約を実施する</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr"/>
@@ -872,14 +772,17 @@
     <row r="43" ht="24" customHeight="1"/>
     <row r="44" ht="24" customHeight="1"/>
     <row r="45" ht="24" customHeight="1">
-      <c r="B45" s="16" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>補足:</t>
         </is>
       </c>
-      <c r="C45" s="17" t="inlineStr">
-        <is>
-          <t>中断したLPN分割作業のうち、未処理の部材のみを対象とする。</t>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>対象：④複数部材をLPN分割する途中で中断した場合
+未処理の部材を親部材へ集約する。
+中断したLPN分割作業のうち、
+未処理の部材のみを対象とすること。</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
@@ -910,15 +813,14 @@
     <row r="49" ht="24" customHeight="1"/>
     <row r="50" ht="24" customHeight="1"/>
     <row r="51" ht="24" customHeight="1">
-      <c r="B51" s="18" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>【⑤対応】MAラベルを再印刷する
-プリンタを設定しないままLPN分割を行った場合、正しいプリンタを設定し、MAラベルを再印刷する。</t>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>MAラベルを再印刷する</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr"/>
@@ -951,14 +853,16 @@
     <row r="55" ht="24" customHeight="1"/>
     <row r="56" ht="24" customHeight="1"/>
     <row r="57" ht="24" customHeight="1">
-      <c r="B57" s="20" t="inlineStr">
+      <c r="B57" s="8" t="inlineStr">
         <is>
           <t>補足:</t>
         </is>
       </c>
-      <c r="C57" s="21" t="inlineStr">
-        <is>
-          <t>再印刷前に旧ラベルを必ず破棄すること。</t>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>対象：⑤プリンタを設定しないままLPN分割した場合
+正しいプリンタを設定し、MAラベルを再印刷する。
+再印刷前に旧ラベルを必ず破棄すること。</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -981,7 +885,7 @@
     <row r="61" ht="24" customHeight="1"/>
     <row r="62" ht="24" customHeight="1"/>
   </sheetData>
-  <mergeCells count="70">
+  <mergeCells count="71">
     <mergeCell ref="C51:H56"/>
     <mergeCell ref="B51:B56"/>
     <mergeCell ref="I39:I50"/>
@@ -1041,19 +945,19 @@
     <mergeCell ref="K9:M11"/>
     <mergeCell ref="J24:J26"/>
     <mergeCell ref="K36:M38"/>
+    <mergeCell ref="B1:T1"/>
     <mergeCell ref="N39:T50"/>
-    <mergeCell ref="K51:M53"/>
     <mergeCell ref="K30:M32"/>
     <mergeCell ref="K45:M47"/>
-    <mergeCell ref="K54:M56"/>
+    <mergeCell ref="K51:M53"/>
     <mergeCell ref="K21:M23"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J54:J56"/>
+    <mergeCell ref="K54:M56"/>
     <mergeCell ref="J27:J29"/>
     <mergeCell ref="C21:H26"/>
     <mergeCell ref="K60:M62"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>